<commit_message>
Updated the changes related to hosting
</commit_message>
<xml_diff>
--- a/Files/Data/Property Portfolio Data.xlsx
+++ b/Files/Data/Property Portfolio Data.xlsx
@@ -5,17 +5,17 @@
   <workbookPr codeName="ThisWorkbook" defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\tmail-merge-with-vue-docx-editor-and-spreadsheet\Files\Data\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\EJ2\Samples\presale_demo\mail-merge-with-vue-docx-editor-and-spreadsheet\Files\Data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AE689D0B-02BA-4D02-BB3C-32CAB74597AF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E548D21C-8AF0-4021-8AC0-7C3B026B3398}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="30936" windowHeight="16776" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Property Information" sheetId="1" r:id="rId1"/>
     <sheet name="Rent Roll Data" sheetId="2" r:id="rId2"/>
-    <sheet name="Appraisal Summary" sheetId="4" r:id="rId3"/>
+    <sheet name="Appraisal Summary" sheetId="3" r:id="rId3"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -241,58 +241,58 @@
     <t>Tenant 6</t>
   </si>
   <si>
+    <t>T007</t>
+  </si>
+  <si>
+    <t>Tenant 7</t>
+  </si>
+  <si>
+    <t>T008</t>
+  </si>
+  <si>
+    <t>Tenant 8</t>
+  </si>
+  <si>
+    <t>Consulting</t>
+  </si>
+  <si>
+    <t>T009</t>
+  </si>
+  <si>
+    <t>Tenant 9</t>
+  </si>
+  <si>
+    <t>Technology</t>
+  </si>
+  <si>
+    <t>T010</t>
+  </si>
+  <si>
+    <t>Tenant 10</t>
+  </si>
+  <si>
+    <t>T011</t>
+  </si>
+  <si>
+    <t>Tenant 11</t>
+  </si>
+  <si>
+    <t>T012</t>
+  </si>
+  <si>
+    <t>Tenant 12</t>
+  </si>
+  <si>
+    <t>T013</t>
+  </si>
+  <si>
+    <t>Tenant 13</t>
+  </si>
+  <si>
+    <t>Marketing</t>
+  </si>
+  <si>
     <t>Vacant</t>
-  </si>
-  <si>
-    <t>T007</t>
-  </si>
-  <si>
-    <t>Tenant 7</t>
-  </si>
-  <si>
-    <t>T008</t>
-  </si>
-  <si>
-    <t>Tenant 8</t>
-  </si>
-  <si>
-    <t>Consulting</t>
-  </si>
-  <si>
-    <t>T009</t>
-  </si>
-  <si>
-    <t>Tenant 9</t>
-  </si>
-  <si>
-    <t>Technology</t>
-  </si>
-  <si>
-    <t>T010</t>
-  </si>
-  <si>
-    <t>Tenant 10</t>
-  </si>
-  <si>
-    <t>T011</t>
-  </si>
-  <si>
-    <t>Tenant 11</t>
-  </si>
-  <si>
-    <t>T012</t>
-  </si>
-  <si>
-    <t>Tenant 12</t>
-  </si>
-  <si>
-    <t>T013</t>
-  </si>
-  <si>
-    <t>Tenant 13</t>
-  </si>
-  <si>
-    <t>Marketing</t>
   </si>
   <si>
     <t>T014</t>
@@ -619,8 +619,8 @@
   </cellStyleXfs>
   <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="164" fontId="2" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="10" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
@@ -638,7 +638,7 @@
     <dxf>
       <fill>
         <patternFill>
-          <fgColor indexed="64"/>
+          <fgColor rgb="FF000000"/>
           <bgColor rgb="FFFFFFFF"/>
         </patternFill>
       </fill>
@@ -956,90 +956,90 @@
   <dimension ref="A1:U2"/>
   <sheetFormatPr defaultRowHeight="14.4" customHeight="1" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="10.5546875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="13.88671875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="23.33203125" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="15.77734375" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="7.44140625" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="5.33203125" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="8.33203125" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="12.33203125" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="23.33203125" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="22.44140625" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="15.88671875" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="15.6640625" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="15.88671875" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="16.44140625" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="17.21875" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="13.21875" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="15.109375" bestFit="1" customWidth="1"/>
-    <col min="19" max="19" width="31" bestFit="1" customWidth="1"/>
-    <col min="20" max="20" width="33.88671875" bestFit="1" customWidth="1"/>
-    <col min="21" max="21" width="17.21875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="10.5546875" customWidth="1"/>
+    <col min="2" max="2" width="13.88671875" customWidth="1"/>
+    <col min="3" max="3" width="23.21875" customWidth="1"/>
+    <col min="4" max="4" width="15.6640625" customWidth="1"/>
+    <col min="5" max="5" width="7.44140625" customWidth="1"/>
+    <col min="6" max="6" width="5.21875" customWidth="1"/>
+    <col min="7" max="7" width="8.21875" customWidth="1"/>
+    <col min="9" max="9" width="12.21875" customWidth="1"/>
+    <col min="10" max="10" width="23.21875" customWidth="1"/>
+    <col min="11" max="11" width="22.44140625" customWidth="1"/>
+    <col min="12" max="12" width="15.88671875" customWidth="1"/>
+    <col min="13" max="13" width="15.6640625" customWidth="1"/>
+    <col min="14" max="14" width="15.88671875" customWidth="1"/>
+    <col min="15" max="15" width="16.44140625" customWidth="1"/>
+    <col min="16" max="16" width="17.21875" customWidth="1"/>
+    <col min="17" max="17" width="13.21875" customWidth="1"/>
+    <col min="18" max="18" width="15.109375" customWidth="1"/>
+    <col min="19" max="19" width="31" customWidth="1"/>
+    <col min="20" max="20" width="33.88671875" customWidth="1"/>
+    <col min="21" max="21" width="17.21875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:21" s="2" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="2" t="s">
+    <row r="1" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="2" t="s">
+      <c r="B1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="2" t="s">
+      <c r="C1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="2" t="s">
+      <c r="D1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="2" t="s">
+      <c r="E1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="2" t="s">
+      <c r="F1" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="2" t="s">
+      <c r="G1" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="2" t="s">
+      <c r="H1" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="2" t="s">
+      <c r="I1" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="2" t="s">
+      <c r="J1" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" s="2" t="s">
+      <c r="K1" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="L1" s="2" t="s">
+      <c r="L1" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="M1" s="2" t="s">
+      <c r="M1" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="N1" s="2" t="s">
+      <c r="N1" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="O1" s="2" t="s">
+      <c r="O1" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="P1" s="2" t="s">
+      <c r="P1" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="Q1" s="2" t="s">
+      <c r="Q1" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="R1" s="2" t="s">
+      <c r="R1" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="S1" s="2" t="s">
+      <c r="S1" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="T1" s="2" t="s">
+      <c r="T1" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="U1" s="2" t="s">
+      <c r="U1" s="1" t="s">
         <v>20</v>
       </c>
     </row>
@@ -1098,10 +1098,10 @@
       <c r="R2">
         <v>6.5000000000000002E-2</v>
       </c>
-      <c r="S2" s="1">
+      <c r="S2" s="2">
         <v>450000</v>
       </c>
-      <c r="T2" s="1">
+      <c r="T2" s="2">
         <v>120000</v>
       </c>
       <c r="U2" t="s">
@@ -1129,28 +1129,28 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:18" x14ac:dyDescent="0.3">
-      <c r="A1" s="2" t="s">
+      <c r="A1" s="1" t="s">
         <v>31</v>
       </c>
-      <c r="B1" s="2" t="s">
+      <c r="B1" s="1" t="s">
         <v>32</v>
       </c>
-      <c r="C1" s="2" t="s">
+      <c r="C1" s="1" t="s">
         <v>33</v>
       </c>
-      <c r="D1" s="2" t="s">
+      <c r="D1" s="1" t="s">
         <v>34</v>
       </c>
-      <c r="E1" s="2" t="s">
+      <c r="E1" s="1" t="s">
         <v>35</v>
       </c>
-      <c r="F1" s="2" t="s">
+      <c r="F1" s="1" t="s">
         <v>36</v>
       </c>
-      <c r="G1" s="2" t="s">
+      <c r="G1" s="1" t="s">
         <v>37</v>
       </c>
-      <c r="H1" s="2" t="s">
+      <c r="H1" s="1" t="s">
         <v>38</v>
       </c>
       <c r="I1" s="3" t="s">
@@ -1165,22 +1165,22 @@
       <c r="L1" s="3" t="s">
         <v>42</v>
       </c>
-      <c r="M1" s="2" t="s">
+      <c r="M1" s="1" t="s">
         <v>43</v>
       </c>
       <c r="N1" s="3" t="s">
         <v>44</v>
       </c>
-      <c r="O1" s="2" t="s">
+      <c r="O1" s="1" t="s">
         <v>45</v>
       </c>
-      <c r="P1" s="2" t="s">
+      <c r="P1" s="1" t="s">
         <v>46</v>
       </c>
-      <c r="Q1" s="2" t="s">
+      <c r="Q1" s="1" t="s">
         <v>47</v>
       </c>
-      <c r="R1" s="2" t="s">
+      <c r="R1" s="1" t="s">
         <v>48</v>
       </c>
     </row>
@@ -1209,23 +1209,23 @@
       <c r="H2">
         <v>3217</v>
       </c>
-      <c r="I2" s="1">
+      <c r="I2" s="2">
         <v>4398</v>
       </c>
-      <c r="J2" s="1">
+      <c r="J2" s="2">
         <v>426</v>
       </c>
-      <c r="K2" s="1">
+      <c r="K2" s="2">
         <f t="shared" ref="K2:K33" si="0">IF(M2="Occupied",I2+J2,0)</f>
         <v>4824</v>
       </c>
-      <c r="L2" s="1">
+      <c r="L2" s="2">
         <v>8796</v>
       </c>
       <c r="M2" t="s">
         <v>52</v>
       </c>
-      <c r="N2" s="1">
+      <c r="N2" s="2">
         <f t="shared" ref="N2:N33" si="1">K2*12</f>
         <v>57888</v>
       </c>
@@ -1265,23 +1265,23 @@
       <c r="H3">
         <v>1145</v>
       </c>
-      <c r="I3" s="1">
+      <c r="I3" s="2">
         <v>5634</v>
       </c>
-      <c r="J3" s="1">
+      <c r="J3" s="2">
         <v>790</v>
       </c>
-      <c r="K3" s="1">
+      <c r="K3" s="2">
         <f t="shared" si="0"/>
         <v>6424</v>
       </c>
-      <c r="L3" s="1">
+      <c r="L3" s="2">
         <v>11268</v>
       </c>
       <c r="M3" t="s">
         <v>52</v>
       </c>
-      <c r="N3" s="1">
+      <c r="N3" s="2">
         <f t="shared" si="1"/>
         <v>77088</v>
       </c>
@@ -1321,23 +1321,23 @@
       <c r="H4">
         <v>2727</v>
       </c>
-      <c r="I4" s="1">
+      <c r="I4" s="2">
         <v>3753</v>
       </c>
-      <c r="J4" s="1">
+      <c r="J4" s="2">
         <v>156</v>
       </c>
-      <c r="K4" s="1">
+      <c r="K4" s="2">
         <f t="shared" si="0"/>
         <v>3909</v>
       </c>
-      <c r="L4" s="1">
+      <c r="L4" s="2">
         <v>7506</v>
       </c>
       <c r="M4" t="s">
         <v>52</v>
       </c>
-      <c r="N4" s="1">
+      <c r="N4" s="2">
         <f t="shared" si="1"/>
         <v>46908</v>
       </c>
@@ -1377,23 +1377,23 @@
       <c r="H5">
         <v>1269</v>
       </c>
-      <c r="I5" s="1">
+      <c r="I5" s="2">
         <v>2768</v>
       </c>
-      <c r="J5" s="1">
+      <c r="J5" s="2">
         <v>280</v>
       </c>
-      <c r="K5" s="1">
+      <c r="K5" s="2">
         <f t="shared" si="0"/>
         <v>3048</v>
       </c>
-      <c r="L5" s="1">
+      <c r="L5" s="2">
         <v>5536</v>
       </c>
       <c r="M5" t="s">
         <v>52</v>
       </c>
-      <c r="N5" s="1">
+      <c r="N5" s="2">
         <f t="shared" si="1"/>
         <v>36576</v>
       </c>
@@ -1433,23 +1433,23 @@
       <c r="H6">
         <v>1571</v>
       </c>
-      <c r="I6" s="1">
+      <c r="I6" s="2">
         <v>4891</v>
       </c>
-      <c r="J6" s="1">
+      <c r="J6" s="2">
         <v>169</v>
       </c>
-      <c r="K6" s="1">
+      <c r="K6" s="2">
         <f t="shared" si="0"/>
         <v>5060</v>
       </c>
-      <c r="L6" s="1">
+      <c r="L6" s="2">
         <v>9782</v>
       </c>
       <c r="M6" t="s">
         <v>52</v>
       </c>
-      <c r="N6" s="1">
+      <c r="N6" s="2">
         <f t="shared" si="1"/>
         <v>60720</v>
       </c>
@@ -1489,23 +1489,23 @@
       <c r="H7">
         <v>1619</v>
       </c>
-      <c r="I7" s="1">
+      <c r="I7" s="2">
         <v>3267</v>
       </c>
-      <c r="J7" s="1">
+      <c r="J7" s="2">
         <v>186</v>
       </c>
-      <c r="K7" s="1">
+      <c r="K7" s="2">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="L7" s="1">
+      <c r="L7" s="2">
         <v>8250</v>
       </c>
       <c r="M7" t="s">
-        <v>68</v>
-      </c>
-      <c r="N7" s="1">
+        <v>85</v>
+      </c>
+      <c r="N7" s="2">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
@@ -1525,10 +1525,10 @@
         <v>7</v>
       </c>
       <c r="B8" t="s">
+        <v>68</v>
+      </c>
+      <c r="C8" t="s">
         <v>69</v>
-      </c>
-      <c r="C8" t="s">
-        <v>70</v>
       </c>
       <c r="D8" t="s">
         <v>63</v>
@@ -1545,23 +1545,23 @@
       <c r="H8">
         <v>3059</v>
       </c>
-      <c r="I8" s="1">
+      <c r="I8" s="2">
         <v>5852</v>
       </c>
-      <c r="J8" s="1">
+      <c r="J8" s="2">
         <v>316</v>
       </c>
-      <c r="K8" s="1">
+      <c r="K8" s="2">
         <f t="shared" si="0"/>
         <v>6168</v>
       </c>
-      <c r="L8" s="1">
+      <c r="L8" s="2">
         <v>11704</v>
       </c>
       <c r="M8" t="s">
         <v>52</v>
       </c>
-      <c r="N8" s="1">
+      <c r="N8" s="2">
         <f t="shared" si="1"/>
         <v>74016</v>
       </c>
@@ -1581,13 +1581,13 @@
         <v>8</v>
       </c>
       <c r="B9" t="s">
+        <v>70</v>
+      </c>
+      <c r="C9" t="s">
         <v>71</v>
       </c>
-      <c r="C9" t="s">
+      <c r="D9" t="s">
         <v>72</v>
-      </c>
-      <c r="D9" t="s">
-        <v>73</v>
       </c>
       <c r="E9" s="4">
         <v>45292</v>
@@ -1601,23 +1601,23 @@
       <c r="H9">
         <v>3257</v>
       </c>
-      <c r="I9" s="1">
+      <c r="I9" s="2">
         <v>2940</v>
       </c>
-      <c r="J9" s="1">
+      <c r="J9" s="2">
         <v>539</v>
       </c>
-      <c r="K9" s="1">
+      <c r="K9" s="2">
         <f t="shared" si="0"/>
         <v>3479</v>
       </c>
-      <c r="L9" s="1">
+      <c r="L9" s="2">
         <v>5880</v>
       </c>
       <c r="M9" t="s">
         <v>52</v>
       </c>
-      <c r="N9" s="1">
+      <c r="N9" s="2">
         <f t="shared" si="1"/>
         <v>41748</v>
       </c>
@@ -1637,13 +1637,13 @@
         <v>9</v>
       </c>
       <c r="B10" t="s">
+        <v>73</v>
+      </c>
+      <c r="C10" t="s">
         <v>74</v>
       </c>
-      <c r="C10" t="s">
+      <c r="D10" t="s">
         <v>75</v>
-      </c>
-      <c r="D10" t="s">
-        <v>76</v>
       </c>
       <c r="E10" s="4">
         <v>45292</v>
@@ -1657,23 +1657,23 @@
       <c r="H10">
         <v>1523</v>
       </c>
-      <c r="I10" s="1">
+      <c r="I10" s="2">
         <v>4339</v>
       </c>
-      <c r="J10" s="1">
+      <c r="J10" s="2">
         <v>798</v>
       </c>
-      <c r="K10" s="1">
+      <c r="K10" s="2">
         <f t="shared" si="0"/>
         <v>5137</v>
       </c>
-      <c r="L10" s="1">
+      <c r="L10" s="2">
         <v>8678</v>
       </c>
       <c r="M10" t="s">
         <v>52</v>
       </c>
-      <c r="N10" s="1">
+      <c r="N10" s="2">
         <f t="shared" si="1"/>
         <v>61644</v>
       </c>
@@ -1693,10 +1693,10 @@
         <v>10</v>
       </c>
       <c r="B11" t="s">
+        <v>76</v>
+      </c>
+      <c r="C11" t="s">
         <v>77</v>
-      </c>
-      <c r="C11" t="s">
-        <v>78</v>
       </c>
       <c r="D11" t="s">
         <v>63</v>
@@ -1713,23 +1713,23 @@
       <c r="H11">
         <v>2788</v>
       </c>
-      <c r="I11" s="1">
+      <c r="I11" s="2">
         <v>4793</v>
       </c>
-      <c r="J11" s="1">
+      <c r="J11" s="2">
         <v>519</v>
       </c>
-      <c r="K11" s="1">
+      <c r="K11" s="2">
         <f t="shared" si="0"/>
         <v>5312</v>
       </c>
-      <c r="L11" s="1">
+      <c r="L11" s="2">
         <v>9586</v>
       </c>
       <c r="M11" t="s">
         <v>52</v>
       </c>
-      <c r="N11" s="1">
+      <c r="N11" s="2">
         <f t="shared" si="1"/>
         <v>63744</v>
       </c>
@@ -1749,10 +1749,10 @@
         <v>11</v>
       </c>
       <c r="B12" t="s">
+        <v>78</v>
+      </c>
+      <c r="C12" t="s">
         <v>79</v>
-      </c>
-      <c r="C12" t="s">
-        <v>80</v>
       </c>
       <c r="D12" t="s">
         <v>56</v>
@@ -1769,23 +1769,23 @@
       <c r="H12">
         <v>2240</v>
       </c>
-      <c r="I12" s="1">
+      <c r="I12" s="2">
         <v>4235</v>
       </c>
-      <c r="J12" s="1">
+      <c r="J12" s="2">
         <v>145</v>
       </c>
-      <c r="K12" s="1">
+      <c r="K12" s="2">
         <f t="shared" si="0"/>
         <v>4380</v>
       </c>
-      <c r="L12" s="1">
+      <c r="L12" s="2">
         <v>8470</v>
       </c>
       <c r="M12" t="s">
         <v>52</v>
       </c>
-      <c r="N12" s="1">
+      <c r="N12" s="2">
         <f t="shared" si="1"/>
         <v>52560</v>
       </c>
@@ -1805,13 +1805,13 @@
         <v>12</v>
       </c>
       <c r="B13" t="s">
+        <v>80</v>
+      </c>
+      <c r="C13" t="s">
         <v>81</v>
       </c>
-      <c r="C13" t="s">
-        <v>82</v>
-      </c>
       <c r="D13" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="E13" s="4">
         <v>45292</v>
@@ -1825,23 +1825,23 @@
       <c r="H13">
         <v>2200</v>
       </c>
-      <c r="I13" s="1">
+      <c r="I13" s="2">
         <v>3756</v>
       </c>
-      <c r="J13" s="1">
+      <c r="J13" s="2">
         <v>698</v>
       </c>
-      <c r="K13" s="1">
+      <c r="K13" s="2">
         <f t="shared" si="0"/>
         <v>4454</v>
       </c>
-      <c r="L13" s="1">
+      <c r="L13" s="2">
         <v>7512</v>
       </c>
       <c r="M13" t="s">
         <v>52</v>
       </c>
-      <c r="N13" s="1">
+      <c r="N13" s="2">
         <f t="shared" si="1"/>
         <v>53448</v>
       </c>
@@ -1861,13 +1861,13 @@
         <v>13</v>
       </c>
       <c r="B14" t="s">
+        <v>82</v>
+      </c>
+      <c r="C14" t="s">
         <v>83</v>
       </c>
-      <c r="C14" t="s">
+      <c r="D14" t="s">
         <v>84</v>
-      </c>
-      <c r="D14" t="s">
-        <v>85</v>
       </c>
       <c r="E14" s="4">
         <v>45292</v>
@@ -1881,23 +1881,23 @@
       <c r="H14">
         <v>1137</v>
       </c>
-      <c r="I14" s="1">
+      <c r="I14" s="2">
         <v>2469</v>
       </c>
-      <c r="J14" s="1">
+      <c r="J14" s="2">
         <v>136</v>
       </c>
-      <c r="K14" s="1">
+      <c r="K14" s="2">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="L14" s="1">
+      <c r="L14" s="2">
         <v>5437</v>
       </c>
       <c r="M14" t="s">
-        <v>68</v>
-      </c>
-      <c r="N14" s="1">
+        <v>85</v>
+      </c>
+      <c r="N14" s="2">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
@@ -1923,7 +1923,7 @@
         <v>87</v>
       </c>
       <c r="D15" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="E15" s="4">
         <v>45292</v>
@@ -1937,23 +1937,23 @@
       <c r="H15">
         <v>1067</v>
       </c>
-      <c r="I15" s="1">
+      <c r="I15" s="2">
         <v>5082</v>
       </c>
-      <c r="J15" s="1">
+      <c r="J15" s="2">
         <v>134</v>
       </c>
-      <c r="K15" s="1">
+      <c r="K15" s="2">
         <f t="shared" si="0"/>
         <v>5216</v>
       </c>
-      <c r="L15" s="1">
+      <c r="L15" s="2">
         <v>10164</v>
       </c>
       <c r="M15" t="s">
         <v>52</v>
       </c>
-      <c r="N15" s="1">
+      <c r="N15" s="2">
         <f t="shared" si="1"/>
         <v>62592</v>
       </c>
@@ -1979,7 +1979,7 @@
         <v>89</v>
       </c>
       <c r="D16" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="E16" s="4">
         <v>45292</v>
@@ -1993,23 +1993,23 @@
       <c r="H16">
         <v>1415</v>
       </c>
-      <c r="I16" s="1">
+      <c r="I16" s="2">
         <v>1909</v>
       </c>
-      <c r="J16" s="1">
+      <c r="J16" s="2">
         <v>629</v>
       </c>
-      <c r="K16" s="1">
+      <c r="K16" s="2">
         <f t="shared" si="0"/>
         <v>2538</v>
       </c>
-      <c r="L16" s="1">
+      <c r="L16" s="2">
         <v>3818</v>
       </c>
       <c r="M16" t="s">
         <v>52</v>
       </c>
-      <c r="N16" s="1">
+      <c r="N16" s="2">
         <f t="shared" si="1"/>
         <v>30456</v>
       </c>
@@ -2035,7 +2035,7 @@
         <v>91</v>
       </c>
       <c r="D17" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="E17" s="4">
         <v>45292</v>
@@ -2049,23 +2049,23 @@
       <c r="H17">
         <v>2885</v>
       </c>
-      <c r="I17" s="1">
+      <c r="I17" s="2">
         <v>5879</v>
       </c>
-      <c r="J17" s="1">
+      <c r="J17" s="2">
         <v>356</v>
       </c>
-      <c r="K17" s="1">
+      <c r="K17" s="2">
         <f t="shared" si="0"/>
         <v>6235</v>
       </c>
-      <c r="L17" s="1">
+      <c r="L17" s="2">
         <v>11758</v>
       </c>
       <c r="M17" t="s">
         <v>52</v>
       </c>
-      <c r="N17" s="1">
+      <c r="N17" s="2">
         <f t="shared" si="1"/>
         <v>74820</v>
       </c>
@@ -2091,7 +2091,7 @@
         <v>93</v>
       </c>
       <c r="D18" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="E18" s="4">
         <v>45292</v>
@@ -2105,23 +2105,23 @@
       <c r="H18">
         <v>1813</v>
       </c>
-      <c r="I18" s="1">
+      <c r="I18" s="2">
         <v>3393</v>
       </c>
-      <c r="J18" s="1">
+      <c r="J18" s="2">
         <v>149</v>
       </c>
-      <c r="K18" s="1">
+      <c r="K18" s="2">
         <f t="shared" si="0"/>
         <v>3542</v>
       </c>
-      <c r="L18" s="1">
+      <c r="L18" s="2">
         <v>6786</v>
       </c>
       <c r="M18" t="s">
         <v>52</v>
       </c>
-      <c r="N18" s="1">
+      <c r="N18" s="2">
         <f t="shared" si="1"/>
         <v>42504</v>
       </c>
@@ -2147,7 +2147,7 @@
         <v>95</v>
       </c>
       <c r="D19" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="E19" s="4">
         <v>45292</v>
@@ -2161,23 +2161,23 @@
       <c r="H19">
         <v>2019</v>
       </c>
-      <c r="I19" s="1">
+      <c r="I19" s="2">
         <v>3011</v>
       </c>
-      <c r="J19" s="1">
+      <c r="J19" s="2">
         <v>796</v>
       </c>
-      <c r="K19" s="1">
+      <c r="K19" s="2">
         <f t="shared" si="0"/>
         <v>3807</v>
       </c>
-      <c r="L19" s="1">
+      <c r="L19" s="2">
         <v>6022</v>
       </c>
       <c r="M19" t="s">
         <v>52</v>
       </c>
-      <c r="N19" s="1">
+      <c r="N19" s="2">
         <f t="shared" si="1"/>
         <v>45684</v>
       </c>
@@ -2217,23 +2217,23 @@
       <c r="H20">
         <v>3026</v>
       </c>
-      <c r="I20" s="1">
+      <c r="I20" s="2">
         <v>4722</v>
       </c>
-      <c r="J20" s="1">
+      <c r="J20" s="2">
         <v>256</v>
       </c>
-      <c r="K20" s="1">
+      <c r="K20" s="2">
         <f t="shared" si="0"/>
         <v>4978</v>
       </c>
-      <c r="L20" s="1">
+      <c r="L20" s="2">
         <v>9444</v>
       </c>
       <c r="M20" t="s">
         <v>52</v>
       </c>
-      <c r="N20" s="1">
+      <c r="N20" s="2">
         <f t="shared" si="1"/>
         <v>59736</v>
       </c>
@@ -2259,7 +2259,7 @@
         <v>99</v>
       </c>
       <c r="D21" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="E21" s="4">
         <v>45292</v>
@@ -2273,23 +2273,23 @@
       <c r="H21">
         <v>2524</v>
       </c>
-      <c r="I21" s="1">
+      <c r="I21" s="2">
         <v>4899</v>
       </c>
-      <c r="J21" s="1">
+      <c r="J21" s="2">
         <v>215</v>
       </c>
-      <c r="K21" s="1">
+      <c r="K21" s="2">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="L21" s="1">
+      <c r="L21" s="2">
         <v>8600</v>
       </c>
       <c r="M21" t="s">
-        <v>68</v>
-      </c>
-      <c r="N21" s="1">
+        <v>85</v>
+      </c>
+      <c r="N21" s="2">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
@@ -2329,23 +2329,23 @@
       <c r="H22">
         <v>3107</v>
       </c>
-      <c r="I22" s="1">
+      <c r="I22" s="2">
         <v>5151</v>
       </c>
-      <c r="J22" s="1">
+      <c r="J22" s="2">
         <v>428</v>
       </c>
-      <c r="K22" s="1">
+      <c r="K22" s="2">
         <f t="shared" si="0"/>
         <v>5579</v>
       </c>
-      <c r="L22" s="1">
+      <c r="L22" s="2">
         <v>10302</v>
       </c>
       <c r="M22" t="s">
         <v>52</v>
       </c>
-      <c r="N22" s="1">
+      <c r="N22" s="2">
         <f t="shared" si="1"/>
         <v>66948</v>
       </c>
@@ -2371,7 +2371,7 @@
         <v>103</v>
       </c>
       <c r="D23" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="E23" s="4">
         <v>45292</v>
@@ -2385,23 +2385,23 @@
       <c r="H23">
         <v>1261</v>
       </c>
-      <c r="I23" s="1">
+      <c r="I23" s="2">
         <v>5618</v>
       </c>
-      <c r="J23" s="1">
+      <c r="J23" s="2">
         <v>551</v>
       </c>
-      <c r="K23" s="1">
+      <c r="K23" s="2">
         <f t="shared" si="0"/>
         <v>6169</v>
       </c>
-      <c r="L23" s="1">
+      <c r="L23" s="2">
         <v>11236</v>
       </c>
       <c r="M23" t="s">
         <v>52</v>
       </c>
-      <c r="N23" s="1">
+      <c r="N23" s="2">
         <f t="shared" si="1"/>
         <v>74028</v>
       </c>
@@ -2441,23 +2441,23 @@
       <c r="H24">
         <v>1268</v>
       </c>
-      <c r="I24" s="1">
+      <c r="I24" s="2">
         <v>5465</v>
       </c>
-      <c r="J24" s="1">
+      <c r="J24" s="2">
         <v>688</v>
       </c>
-      <c r="K24" s="1">
+      <c r="K24" s="2">
         <f t="shared" si="0"/>
         <v>6153</v>
       </c>
-      <c r="L24" s="1">
+      <c r="L24" s="2">
         <v>10930</v>
       </c>
       <c r="M24" t="s">
         <v>52</v>
       </c>
-      <c r="N24" s="1">
+      <c r="N24" s="2">
         <f t="shared" si="1"/>
         <v>73836</v>
       </c>
@@ -2497,23 +2497,23 @@
       <c r="H25">
         <v>2559</v>
       </c>
-      <c r="I25" s="1">
+      <c r="I25" s="2">
         <v>2678</v>
       </c>
-      <c r="J25" s="1">
+      <c r="J25" s="2">
         <v>607</v>
       </c>
-      <c r="K25" s="1">
+      <c r="K25" s="2">
         <f t="shared" si="0"/>
         <v>3285</v>
       </c>
-      <c r="L25" s="1">
+      <c r="L25" s="2">
         <v>5356</v>
       </c>
       <c r="M25" t="s">
         <v>52</v>
       </c>
-      <c r="N25" s="1">
+      <c r="N25" s="2">
         <f t="shared" si="1"/>
         <v>39420</v>
       </c>
@@ -2539,7 +2539,7 @@
         <v>109</v>
       </c>
       <c r="D26" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="E26" s="4">
         <v>45292</v>
@@ -2553,23 +2553,23 @@
       <c r="H26">
         <v>1017</v>
       </c>
-      <c r="I26" s="1">
+      <c r="I26" s="2">
         <v>5719</v>
       </c>
-      <c r="J26" s="1">
+      <c r="J26" s="2">
         <v>591</v>
       </c>
-      <c r="K26" s="1">
+      <c r="K26" s="2">
         <f t="shared" si="0"/>
         <v>6310</v>
       </c>
-      <c r="L26" s="1">
+      <c r="L26" s="2">
         <v>11438</v>
       </c>
       <c r="M26" t="s">
         <v>52</v>
       </c>
-      <c r="N26" s="1">
+      <c r="N26" s="2">
         <f t="shared" si="1"/>
         <v>75720</v>
       </c>
@@ -2609,23 +2609,23 @@
       <c r="H27">
         <v>3351</v>
       </c>
-      <c r="I27" s="1">
+      <c r="I27" s="2">
         <v>1964</v>
       </c>
-      <c r="J27" s="1">
+      <c r="J27" s="2">
         <v>571</v>
       </c>
-      <c r="K27" s="1">
+      <c r="K27" s="2">
         <f t="shared" si="0"/>
         <v>2535</v>
       </c>
-      <c r="L27" s="1">
+      <c r="L27" s="2">
         <v>3928</v>
       </c>
       <c r="M27" t="s">
         <v>52</v>
       </c>
-      <c r="N27" s="1">
+      <c r="N27" s="2">
         <f t="shared" si="1"/>
         <v>30420</v>
       </c>
@@ -2651,7 +2651,7 @@
         <v>113</v>
       </c>
       <c r="D28" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="E28" s="4">
         <v>45292</v>
@@ -2665,23 +2665,23 @@
       <c r="H28">
         <v>2306</v>
       </c>
-      <c r="I28" s="1">
+      <c r="I28" s="2">
         <v>5215</v>
       </c>
-      <c r="J28" s="1">
+      <c r="J28" s="2">
         <v>269</v>
       </c>
-      <c r="K28" s="1">
+      <c r="K28" s="2">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="L28" s="1">
+      <c r="L28" s="2">
         <v>8125</v>
       </c>
       <c r="M28" t="s">
-        <v>68</v>
-      </c>
-      <c r="N28" s="1">
+        <v>85</v>
+      </c>
+      <c r="N28" s="2">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
@@ -2707,7 +2707,7 @@
         <v>115</v>
       </c>
       <c r="D29" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="E29" s="4">
         <v>45292</v>
@@ -2721,23 +2721,23 @@
       <c r="H29">
         <v>2895</v>
       </c>
-      <c r="I29" s="1">
+      <c r="I29" s="2">
         <v>2248</v>
       </c>
-      <c r="J29" s="1">
+      <c r="J29" s="2">
         <v>708</v>
       </c>
-      <c r="K29" s="1">
+      <c r="K29" s="2">
         <f t="shared" si="0"/>
         <v>2956</v>
       </c>
-      <c r="L29" s="1">
+      <c r="L29" s="2">
         <v>4496</v>
       </c>
       <c r="M29" t="s">
         <v>52</v>
       </c>
-      <c r="N29" s="1">
+      <c r="N29" s="2">
         <f t="shared" si="1"/>
         <v>35472</v>
       </c>
@@ -2777,23 +2777,23 @@
       <c r="H30">
         <v>1664</v>
       </c>
-      <c r="I30" s="1">
+      <c r="I30" s="2">
         <v>2946</v>
       </c>
-      <c r="J30" s="1">
+      <c r="J30" s="2">
         <v>219</v>
       </c>
-      <c r="K30" s="1">
+      <c r="K30" s="2">
         <f t="shared" si="0"/>
         <v>3165</v>
       </c>
-      <c r="L30" s="1">
+      <c r="L30" s="2">
         <v>5892</v>
       </c>
       <c r="M30" t="s">
         <v>52</v>
       </c>
-      <c r="N30" s="1">
+      <c r="N30" s="2">
         <f t="shared" si="1"/>
         <v>37980</v>
       </c>
@@ -2833,23 +2833,23 @@
       <c r="H31">
         <v>2127</v>
       </c>
-      <c r="I31" s="1">
+      <c r="I31" s="2">
         <v>5614</v>
       </c>
-      <c r="J31" s="1">
+      <c r="J31" s="2">
         <v>584</v>
       </c>
-      <c r="K31" s="1">
+      <c r="K31" s="2">
         <f t="shared" si="0"/>
         <v>6198</v>
       </c>
-      <c r="L31" s="1">
+      <c r="L31" s="2">
         <v>11228</v>
       </c>
       <c r="M31" t="s">
         <v>52</v>
       </c>
-      <c r="N31" s="1">
+      <c r="N31" s="2">
         <f t="shared" si="1"/>
         <v>74376</v>
       </c>
@@ -2889,23 +2889,23 @@
       <c r="H32">
         <v>3043</v>
       </c>
-      <c r="I32" s="1">
+      <c r="I32" s="2">
         <v>2409</v>
       </c>
-      <c r="J32" s="1">
+      <c r="J32" s="2">
         <v>711</v>
       </c>
-      <c r="K32" s="1">
+      <c r="K32" s="2">
         <f t="shared" si="0"/>
         <v>3120</v>
       </c>
-      <c r="L32" s="1">
+      <c r="L32" s="2">
         <v>4818</v>
       </c>
       <c r="M32" t="s">
         <v>52</v>
       </c>
-      <c r="N32" s="1">
+      <c r="N32" s="2">
         <f t="shared" si="1"/>
         <v>37440</v>
       </c>
@@ -2931,7 +2931,7 @@
         <v>123</v>
       </c>
       <c r="D33" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="E33" s="4">
         <v>45292</v>
@@ -2945,23 +2945,23 @@
       <c r="H33">
         <v>804</v>
       </c>
-      <c r="I33" s="1">
+      <c r="I33" s="2">
         <v>3992</v>
       </c>
-      <c r="J33" s="1">
+      <c r="J33" s="2">
         <v>226</v>
       </c>
-      <c r="K33" s="1">
+      <c r="K33" s="2">
         <f t="shared" si="0"/>
         <v>4218</v>
       </c>
-      <c r="L33" s="1">
+      <c r="L33" s="2">
         <v>7984</v>
       </c>
       <c r="M33" t="s">
         <v>52</v>
       </c>
-      <c r="N33" s="1">
+      <c r="N33" s="2">
         <f t="shared" si="1"/>
         <v>50616</v>
       </c>
@@ -3001,23 +3001,23 @@
       <c r="H34">
         <v>886</v>
       </c>
-      <c r="I34" s="1">
+      <c r="I34" s="2">
         <v>5631</v>
       </c>
-      <c r="J34" s="1">
+      <c r="J34" s="2">
         <v>579</v>
       </c>
-      <c r="K34" s="1">
-        <f t="shared" ref="K34:K51" si="3">IF(M34="Occupied",I34+J34,0)</f>
+      <c r="K34" s="2">
+        <f t="shared" ref="K34:K65" si="3">IF(M34="Occupied",I34+J34,0)</f>
         <v>6210</v>
       </c>
-      <c r="L34" s="1">
+      <c r="L34" s="2">
         <v>11262</v>
       </c>
       <c r="M34" t="s">
         <v>52</v>
       </c>
-      <c r="N34" s="1">
+      <c r="N34" s="2">
         <f t="shared" ref="N34:N51" si="4">K34*12</f>
         <v>74520</v>
       </c>
@@ -3043,7 +3043,7 @@
         <v>127</v>
       </c>
       <c r="D35" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="E35" s="4">
         <v>45292</v>
@@ -3057,23 +3057,23 @@
       <c r="H35">
         <v>2111</v>
       </c>
-      <c r="I35" s="1">
+      <c r="I35" s="2">
         <v>4999</v>
       </c>
-      <c r="J35" s="1">
+      <c r="J35" s="2">
         <v>299</v>
       </c>
-      <c r="K35" s="1">
+      <c r="K35" s="2">
         <f t="shared" si="3"/>
         <v>0</v>
       </c>
-      <c r="L35" s="1">
+      <c r="L35" s="2">
         <v>7599</v>
       </c>
       <c r="M35" t="s">
-        <v>68</v>
-      </c>
-      <c r="N35" s="1">
+        <v>85</v>
+      </c>
+      <c r="N35" s="2">
         <f t="shared" si="4"/>
         <v>0</v>
       </c>
@@ -3113,23 +3113,23 @@
       <c r="H36">
         <v>1222</v>
       </c>
-      <c r="I36" s="1">
+      <c r="I36" s="2">
         <v>3236</v>
       </c>
-      <c r="J36" s="1">
+      <c r="J36" s="2">
         <v>241</v>
       </c>
-      <c r="K36" s="1">
+      <c r="K36" s="2">
         <f t="shared" si="3"/>
         <v>3477</v>
       </c>
-      <c r="L36" s="1">
+      <c r="L36" s="2">
         <v>6472</v>
       </c>
       <c r="M36" t="s">
         <v>52</v>
       </c>
-      <c r="N36" s="1">
+      <c r="N36" s="2">
         <f t="shared" si="4"/>
         <v>41724</v>
       </c>
@@ -3155,7 +3155,7 @@
         <v>131</v>
       </c>
       <c r="D37" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="E37" s="4">
         <v>45292</v>
@@ -3169,23 +3169,23 @@
       <c r="H37">
         <v>2411</v>
       </c>
-      <c r="I37" s="1">
+      <c r="I37" s="2">
         <v>3781</v>
       </c>
-      <c r="J37" s="1">
+      <c r="J37" s="2">
         <v>784</v>
       </c>
-      <c r="K37" s="1">
+      <c r="K37" s="2">
         <f t="shared" si="3"/>
         <v>4565</v>
       </c>
-      <c r="L37" s="1">
+      <c r="L37" s="2">
         <v>7562</v>
       </c>
       <c r="M37" t="s">
         <v>52</v>
       </c>
-      <c r="N37" s="1">
+      <c r="N37" s="2">
         <f t="shared" si="4"/>
         <v>54780</v>
       </c>
@@ -3211,7 +3211,7 @@
         <v>133</v>
       </c>
       <c r="D38" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="E38" s="4">
         <v>45292</v>
@@ -3225,23 +3225,23 @@
       <c r="H38">
         <v>1213</v>
       </c>
-      <c r="I38" s="1">
+      <c r="I38" s="2">
         <v>3249</v>
       </c>
-      <c r="J38" s="1">
+      <c r="J38" s="2">
         <v>554</v>
       </c>
-      <c r="K38" s="1">
+      <c r="K38" s="2">
         <f t="shared" si="3"/>
         <v>3803</v>
       </c>
-      <c r="L38" s="1">
+      <c r="L38" s="2">
         <v>6498</v>
       </c>
       <c r="M38" t="s">
         <v>52</v>
       </c>
-      <c r="N38" s="1">
+      <c r="N38" s="2">
         <f t="shared" si="4"/>
         <v>45636</v>
       </c>
@@ -3281,23 +3281,23 @@
       <c r="H39">
         <v>1416</v>
       </c>
-      <c r="I39" s="1">
+      <c r="I39" s="2">
         <v>4355</v>
       </c>
-      <c r="J39" s="1">
+      <c r="J39" s="2">
         <v>104</v>
       </c>
-      <c r="K39" s="1">
+      <c r="K39" s="2">
         <f t="shared" si="3"/>
         <v>4459</v>
       </c>
-      <c r="L39" s="1">
+      <c r="L39" s="2">
         <v>8710</v>
       </c>
       <c r="M39" t="s">
         <v>52</v>
       </c>
-      <c r="N39" s="1">
+      <c r="N39" s="2">
         <f t="shared" si="4"/>
         <v>53508</v>
       </c>
@@ -3323,7 +3323,7 @@
         <v>137</v>
       </c>
       <c r="D40" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="E40" s="4">
         <v>45292</v>
@@ -3337,23 +3337,23 @@
       <c r="H40">
         <v>1716</v>
       </c>
-      <c r="I40" s="1">
+      <c r="I40" s="2">
         <v>3745</v>
       </c>
-      <c r="J40" s="1">
+      <c r="J40" s="2">
         <v>368</v>
       </c>
-      <c r="K40" s="1">
+      <c r="K40" s="2">
         <f t="shared" si="3"/>
         <v>4113</v>
       </c>
-      <c r="L40" s="1">
+      <c r="L40" s="2">
         <v>7490</v>
       </c>
       <c r="M40" t="s">
         <v>52</v>
       </c>
-      <c r="N40" s="1">
+      <c r="N40" s="2">
         <f t="shared" si="4"/>
         <v>49356</v>
       </c>
@@ -3393,23 +3393,23 @@
       <c r="H41">
         <v>3042</v>
       </c>
-      <c r="I41" s="1">
+      <c r="I41" s="2">
         <v>2928</v>
       </c>
-      <c r="J41" s="1">
+      <c r="J41" s="2">
         <v>756</v>
       </c>
-      <c r="K41" s="1">
+      <c r="K41" s="2">
         <f t="shared" si="3"/>
         <v>3684</v>
       </c>
-      <c r="L41" s="1">
+      <c r="L41" s="2">
         <v>5856</v>
       </c>
       <c r="M41" t="s">
         <v>52</v>
       </c>
-      <c r="N41" s="1">
+      <c r="N41" s="2">
         <f t="shared" si="4"/>
         <v>44208</v>
       </c>
@@ -3435,7 +3435,7 @@
         <v>141</v>
       </c>
       <c r="D42" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="E42" s="4">
         <v>45292</v>
@@ -3449,23 +3449,23 @@
       <c r="H42">
         <v>2807</v>
       </c>
-      <c r="I42" s="1">
+      <c r="I42" s="2">
         <v>5988</v>
       </c>
-      <c r="J42" s="1">
+      <c r="J42" s="2">
         <v>266</v>
       </c>
-      <c r="K42" s="1">
+      <c r="K42" s="2">
         <f t="shared" si="3"/>
         <v>0</v>
       </c>
-      <c r="L42" s="1">
+      <c r="L42" s="2">
         <v>8122</v>
       </c>
       <c r="M42" t="s">
-        <v>68</v>
-      </c>
-      <c r="N42" s="1">
+        <v>85</v>
+      </c>
+      <c r="N42" s="2">
         <f t="shared" si="4"/>
         <v>0</v>
       </c>
@@ -3491,7 +3491,7 @@
         <v>143</v>
       </c>
       <c r="D43" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="E43" s="4">
         <v>45292</v>
@@ -3505,23 +3505,23 @@
       <c r="H43">
         <v>1856</v>
       </c>
-      <c r="I43" s="1">
+      <c r="I43" s="2">
         <v>2347</v>
       </c>
-      <c r="J43" s="1">
+      <c r="J43" s="2">
         <v>654</v>
       </c>
-      <c r="K43" s="1">
+      <c r="K43" s="2">
         <f t="shared" si="3"/>
         <v>3001</v>
       </c>
-      <c r="L43" s="1">
+      <c r="L43" s="2">
         <v>4694</v>
       </c>
       <c r="M43" t="s">
         <v>52</v>
       </c>
-      <c r="N43" s="1">
+      <c r="N43" s="2">
         <f t="shared" si="4"/>
         <v>36012</v>
       </c>
@@ -3561,23 +3561,23 @@
       <c r="H44">
         <v>1118</v>
       </c>
-      <c r="I44" s="1">
+      <c r="I44" s="2">
         <v>5404</v>
       </c>
-      <c r="J44" s="1">
+      <c r="J44" s="2">
         <v>720</v>
       </c>
-      <c r="K44" s="1">
+      <c r="K44" s="2">
         <f t="shared" si="3"/>
         <v>6124</v>
       </c>
-      <c r="L44" s="1">
+      <c r="L44" s="2">
         <v>10808</v>
       </c>
       <c r="M44" t="s">
         <v>52</v>
       </c>
-      <c r="N44" s="1">
+      <c r="N44" s="2">
         <f t="shared" si="4"/>
         <v>73488</v>
       </c>
@@ -3617,23 +3617,23 @@
       <c r="H45">
         <v>2542</v>
       </c>
-      <c r="I45" s="1">
+      <c r="I45" s="2">
         <v>2244</v>
       </c>
-      <c r="J45" s="1">
+      <c r="J45" s="2">
         <v>252</v>
       </c>
-      <c r="K45" s="1">
+      <c r="K45" s="2">
         <f t="shared" si="3"/>
         <v>2496</v>
       </c>
-      <c r="L45" s="1">
+      <c r="L45" s="2">
         <v>4488</v>
       </c>
       <c r="M45" t="s">
         <v>52</v>
       </c>
-      <c r="N45" s="1">
+      <c r="N45" s="2">
         <f t="shared" si="4"/>
         <v>29952</v>
       </c>
@@ -3659,7 +3659,7 @@
         <v>149</v>
       </c>
       <c r="D46" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="E46" s="4">
         <v>45292</v>
@@ -3673,23 +3673,23 @@
       <c r="H46">
         <v>887</v>
       </c>
-      <c r="I46" s="1">
+      <c r="I46" s="2">
         <v>5607</v>
       </c>
-      <c r="J46" s="1">
+      <c r="J46" s="2">
         <v>546</v>
       </c>
-      <c r="K46" s="1">
+      <c r="K46" s="2">
         <f t="shared" si="3"/>
         <v>6153</v>
       </c>
-      <c r="L46" s="1">
+      <c r="L46" s="2">
         <v>11214</v>
       </c>
       <c r="M46" t="s">
         <v>52</v>
       </c>
-      <c r="N46" s="1">
+      <c r="N46" s="2">
         <f t="shared" si="4"/>
         <v>73836</v>
       </c>
@@ -3729,23 +3729,23 @@
       <c r="H47">
         <v>3203</v>
       </c>
-      <c r="I47" s="1">
+      <c r="I47" s="2">
         <v>5340</v>
       </c>
-      <c r="J47" s="1">
+      <c r="J47" s="2">
         <v>437</v>
       </c>
-      <c r="K47" s="1">
+      <c r="K47" s="2">
         <f t="shared" si="3"/>
         <v>5777</v>
       </c>
-      <c r="L47" s="1">
+      <c r="L47" s="2">
         <v>10680</v>
       </c>
       <c r="M47" t="s">
         <v>52</v>
       </c>
-      <c r="N47" s="1">
+      <c r="N47" s="2">
         <f t="shared" si="4"/>
         <v>69324</v>
       </c>
@@ -3771,7 +3771,7 @@
         <v>153</v>
       </c>
       <c r="D48" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="E48" s="4">
         <v>45292</v>
@@ -3785,23 +3785,23 @@
       <c r="H48">
         <v>2490</v>
       </c>
-      <c r="I48" s="1">
+      <c r="I48" s="2">
         <v>4870</v>
       </c>
-      <c r="J48" s="1">
+      <c r="J48" s="2">
         <v>437</v>
       </c>
-      <c r="K48" s="1">
+      <c r="K48" s="2">
         <f t="shared" si="3"/>
         <v>5307</v>
       </c>
-      <c r="L48" s="1">
+      <c r="L48" s="2">
         <v>9740</v>
       </c>
       <c r="M48" t="s">
         <v>52</v>
       </c>
-      <c r="N48" s="1">
+      <c r="N48" s="2">
         <f t="shared" si="4"/>
         <v>63684</v>
       </c>
@@ -3827,7 +3827,7 @@
         <v>155</v>
       </c>
       <c r="D49" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="E49" s="4">
         <v>45292</v>
@@ -3841,23 +3841,23 @@
       <c r="H49">
         <v>2883</v>
       </c>
-      <c r="I49" s="1">
+      <c r="I49" s="2">
         <v>4988</v>
       </c>
-      <c r="J49" s="1">
+      <c r="J49" s="2">
         <v>275</v>
       </c>
-      <c r="K49" s="1">
+      <c r="K49" s="2">
         <f t="shared" si="3"/>
         <v>0</v>
       </c>
-      <c r="L49" s="1">
+      <c r="L49" s="2">
         <v>7899</v>
       </c>
       <c r="M49" t="s">
-        <v>68</v>
-      </c>
-      <c r="N49" s="1">
+        <v>85</v>
+      </c>
+      <c r="N49" s="2">
         <f t="shared" si="4"/>
         <v>0</v>
       </c>
@@ -3883,7 +3883,7 @@
         <v>157</v>
       </c>
       <c r="D50" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="E50" s="4">
         <v>45292</v>
@@ -3897,23 +3897,23 @@
       <c r="H50">
         <v>2181</v>
       </c>
-      <c r="I50" s="1">
+      <c r="I50" s="2">
         <v>2059</v>
       </c>
-      <c r="J50" s="1">
+      <c r="J50" s="2">
         <v>514</v>
       </c>
-      <c r="K50" s="1">
+      <c r="K50" s="2">
         <f t="shared" si="3"/>
         <v>2573</v>
       </c>
-      <c r="L50" s="1">
+      <c r="L50" s="2">
         <v>4118</v>
       </c>
       <c r="M50" t="s">
         <v>52</v>
       </c>
-      <c r="N50" s="1">
+      <c r="N50" s="2">
         <f t="shared" si="4"/>
         <v>30876</v>
       </c>
@@ -3953,23 +3953,23 @@
       <c r="H51">
         <v>966</v>
       </c>
-      <c r="I51" s="1">
+      <c r="I51" s="2">
         <v>4890</v>
       </c>
-      <c r="J51" s="1">
+      <c r="J51" s="2">
         <v>308</v>
       </c>
-      <c r="K51" s="1">
+      <c r="K51" s="2">
         <f t="shared" si="3"/>
         <v>5198</v>
       </c>
-      <c r="L51" s="1">
+      <c r="L51" s="2">
         <v>9780</v>
       </c>
       <c r="M51" t="s">
         <v>52</v>
       </c>
-      <c r="N51" s="1">
+      <c r="N51" s="2">
         <f t="shared" si="4"/>
         <v>62376</v>
       </c>
@@ -3996,63 +3996,63 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F8924A27-8E13-4836-A9ED-5420714EE9B4}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="A1:M2"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="14.4" customHeight="1" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="9.88671875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="13.33203125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="11.33203125" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="19.6640625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="16.77734375" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="15.5546875" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="19.21875" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="14.44140625" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="17.44140625" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="17" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="19.77734375" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="12.44140625" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="13.6640625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="9.88671875" customWidth="1"/>
+    <col min="2" max="2" width="13.21875" customWidth="1"/>
+    <col min="3" max="3" width="11.21875" customWidth="1"/>
+    <col min="4" max="4" width="19.6640625" customWidth="1"/>
+    <col min="5" max="5" width="16.6640625" customWidth="1"/>
+    <col min="6" max="6" width="15.5546875" customWidth="1"/>
+    <col min="7" max="7" width="19.21875" customWidth="1"/>
+    <col min="8" max="8" width="14.44140625" customWidth="1"/>
+    <col min="9" max="9" width="17.44140625" customWidth="1"/>
+    <col min="10" max="10" width="17" customWidth="1"/>
+    <col min="11" max="11" width="19.6640625" customWidth="1"/>
+    <col min="12" max="12" width="12.44140625" customWidth="1"/>
+    <col min="13" max="13" width="13.6640625" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="A1" s="2" t="s">
+      <c r="A1" s="1" t="s">
         <v>160</v>
       </c>
-      <c r="B1" s="2" t="s">
+      <c r="B1" s="1" t="s">
         <v>161</v>
       </c>
-      <c r="C1" s="2" t="s">
+      <c r="C1" s="1" t="s">
         <v>162</v>
       </c>
-      <c r="D1" s="2" t="s">
+      <c r="D1" s="1" t="s">
         <v>163</v>
       </c>
-      <c r="E1" s="2" t="s">
+      <c r="E1" s="1" t="s">
         <v>164</v>
       </c>
-      <c r="F1" s="2" t="s">
+      <c r="F1" s="1" t="s">
         <v>165</v>
       </c>
-      <c r="G1" s="2" t="s">
+      <c r="G1" s="1" t="s">
         <v>166</v>
       </c>
-      <c r="H1" s="2" t="s">
+      <c r="H1" s="1" t="s">
         <v>167</v>
       </c>
-      <c r="I1" s="2" t="s">
+      <c r="I1" s="1" t="s">
         <v>168</v>
       </c>
-      <c r="J1" s="2" t="s">
+      <c r="J1" s="1" t="s">
         <v>169</v>
       </c>
-      <c r="K1" s="2" t="s">
+      <c r="K1" s="1" t="s">
         <v>170</v>
       </c>
-      <c r="L1" s="2" t="s">
+      <c r="L1" s="1" t="s">
         <v>171</v>
       </c>
-      <c r="M1" s="2" t="s">
+      <c r="M1" s="1" t="s">
         <v>172</v>
       </c>
     </row>
@@ -4073,15 +4073,15 @@
         <f>B2/A2</f>
         <v>0.86</v>
       </c>
-      <c r="E2" s="1">
+      <c r="E2" s="2">
         <f>SUM('Rent Roll Data'!K2:K51)</f>
         <v>195139</v>
       </c>
-      <c r="F2" s="1">
+      <c r="F2" s="2">
         <f>SUM('Rent Roll Data'!N2:N51)</f>
         <v>2341668</v>
       </c>
-      <c r="G2" s="1">
+      <c r="G2" s="2">
         <f ca="1">AVERAGE('Rent Roll Data'!A11:AX11)</f>
         <v>14934.408333333333</v>
       </c>
@@ -4089,28 +4089,29 @@
         <f>MAX('Rent Roll Data'!H2:H51)</f>
         <v>3351</v>
       </c>
-      <c r="I2" s="1">
+      <c r="I2" s="2">
         <f>MAX('Rent Roll Data'!N2:N51)</f>
         <v>77088</v>
       </c>
-      <c r="J2" s="1">
+      <c r="J2" s="2">
         <f>'Property Information'!S2</f>
         <v>450000</v>
       </c>
-      <c r="K2" s="1">
+      <c r="K2" s="2">
         <f>'Property Information'!T2</f>
         <v>120000</v>
       </c>
-      <c r="L2" s="1">
+      <c r="L2" s="2">
         <f>F2-(J2+K2)</f>
         <v>1771668</v>
       </c>
-      <c r="M2" s="1">
+      <c r="M2" s="2">
         <f>L2/'Property Information'!R2</f>
         <v>27256430.769230768</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <headerFooter alignWithMargins="0"/>
 </worksheet>
 </file>
</xml_diff>